<commit_message>
Retain observed per-column Excel number formats in masked fixtures
</commit_message>
<xml_diff>
--- a/staging/imile-management/reports/fixtures/MASKED_inhub.xlsx
+++ b/staging/imile-management/reports/fixtures/MASKED_inhub.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R3cd0e680eee748df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R9dd16e5c6ab7403b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,8 +13,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
+  <x:numFmts count="2">
     <x:numFmt numFmtId="200" formatCode="General"/>
+    <x:numFmt numFmtId="201" formatCode="@"/>
   </x:numFmts>
   <x:fonts count="1">
     <x:font>
@@ -47,7 +48,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="4">
+  <x:cellXfs count="5">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
@@ -56,6 +57,9 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -396,10 +400,10 @@
       <x:c r="I2" s="3" t="str">
         <x:v>DS(SYN_AKE)</x:v>
       </x:c>
-      <x:c r="J2" s="3" t="str">
-        <x:v>MASKED</x:v>
-      </x:c>
-      <x:c r="K2" s="3" t="str">
+      <x:c r="J2" s="4" t="str">
+        <x:v>MASKED</x:v>
+      </x:c>
+      <x:c r="K2" s="4" t="str">
         <x:v>2099-05-31</x:v>
       </x:c>
       <x:c r="L2" s="3" t="str">
@@ -414,16 +418,16 @@
       <x:c r="O2" s="3" t="str">
         <x:v>2099-05-31 12:34:56</x:v>
       </x:c>
-      <x:c r="P2" s="3" t="str">
+      <x:c r="P2" s="4" t="str">
         <x:v>2099-05-31 12:34:56</x:v>
       </x:c>
-      <x:c r="Q2" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="R2" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S2" s="3" t="str">
+      <x:c r="Q2" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R2" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S2" s="4" t="str">
         <x:v>MASKED</x:v>
       </x:c>
       <x:c r="T2" s="3" t="str">
@@ -476,10 +480,10 @@
       <x:c r="I3" s="3" t="str">
         <x:v>DS(SYN_AKE)</x:v>
       </x:c>
-      <x:c r="J3" s="3" t="str">
-        <x:v>MASKED</x:v>
-      </x:c>
-      <x:c r="K3" s="3" t="str">
+      <x:c r="J3" s="4" t="str">
+        <x:v>MASKED</x:v>
+      </x:c>
+      <x:c r="K3" s="4" t="str">
         <x:v>2099-06-01</x:v>
       </x:c>
       <x:c r="L3" s="3" t="str">
@@ -494,16 +498,16 @@
       <x:c r="O3" s="3" t="str">
         <x:v>2099-06-01 12:34:56</x:v>
       </x:c>
-      <x:c r="P3" s="3" t="str">
-        <x:v>2099-06-01 12:34:56</x:v>
-      </x:c>
-      <x:c r="Q3" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="R3" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S3" s="3" t="str">
+      <x:c r="P3" s="4" t="str">
+        <x:v>2099-06-01 12:34:56</x:v>
+      </x:c>
+      <x:c r="Q3" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R3" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S3" s="4" t="str">
         <x:v>MASKED</x:v>
       </x:c>
       <x:c r="T3" s="3" t="str">
@@ -556,10 +560,10 @@
       <x:c r="I4" s="3" t="str">
         <x:v>DS(SYN_AKE)</x:v>
       </x:c>
-      <x:c r="J4" s="3" t="str">
-        <x:v>MASKED</x:v>
-      </x:c>
-      <x:c r="K4" s="3" t="str">
+      <x:c r="J4" s="4" t="str">
+        <x:v>MASKED</x:v>
+      </x:c>
+      <x:c r="K4" s="4" t="str">
         <x:v>2099-06-01</x:v>
       </x:c>
       <x:c r="L4" s="3" t="str">
@@ -574,16 +578,16 @@
       <x:c r="O4" s="3" t="str">
         <x:v>2099-06-01 12:34:56</x:v>
       </x:c>
-      <x:c r="P4" s="3" t="str">
-        <x:v>2099-06-01 12:34:56</x:v>
-      </x:c>
-      <x:c r="Q4" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="R4" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S4" s="3" t="str">
+      <x:c r="P4" s="4" t="str">
+        <x:v>2099-06-01 12:34:56</x:v>
+      </x:c>
+      <x:c r="Q4" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R4" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S4" s="4" t="str">
         <x:v>MASKED</x:v>
       </x:c>
       <x:c r="T4" s="3" t="str">
@@ -636,10 +640,10 @@
       <x:c r="I5" s="3" t="str">
         <x:v>DS(SYN_AKE)</x:v>
       </x:c>
-      <x:c r="J5" s="3" t="str">
-        <x:v>MASKED</x:v>
-      </x:c>
-      <x:c r="K5" s="3" t="str">
+      <x:c r="J5" s="4" t="str">
+        <x:v>MASKED</x:v>
+      </x:c>
+      <x:c r="K5" s="4" t="str">
         <x:v>2099-06-01</x:v>
       </x:c>
       <x:c r="L5" s="3" t="str">
@@ -654,16 +658,16 @@
       <x:c r="O5" s="3" t="str">
         <x:v>2099-06-01 12:34:56</x:v>
       </x:c>
-      <x:c r="P5" s="3" t="str">
-        <x:v>2099-06-01 12:34:56</x:v>
-      </x:c>
-      <x:c r="Q5" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="R5" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S5" s="3" t="str">
+      <x:c r="P5" s="4" t="str">
+        <x:v>2099-06-01 12:34:56</x:v>
+      </x:c>
+      <x:c r="Q5" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R5" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S5" s="4" t="str">
         <x:v>MASKED</x:v>
       </x:c>
       <x:c r="T5" s="3" t="str">

</xml_diff>